<commit_message>
Group A hand map: 6807 / 6803 / 5602 / 5604 / 6503 mapped by hand, promote-test fix -> stage now 31 new configurations
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PJcT2926CUEincCxCV1ZSx
</commit_message>
<xml_diff>
--- a/tools/_out/brennancad_20261021/regen/stage/straight/DesignTable_5405_SW2.xlsx
+++ b/tools/_out/brennancad_20261021/regen/stage/straight/DesignTable_5405_SW2.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF33"/>
+  <dimension ref="A1:AF34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3780,83 +3780,83 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>5405-24-20</t>
+          <t>5405-20-32</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>2.54</v>
+        <v>2.6</v>
       </c>
       <c r="C30" t="n">
-        <v>1.1547</v>
+        <v>1.65988</v>
       </c>
       <c r="D30" t="n">
-        <v>2</v>
+        <v>2.875</v>
       </c>
       <c r="E30" t="n">
-        <v>0.93283</v>
+        <v>0.81335</v>
       </c>
       <c r="F30" t="n">
-        <v>0.7235</v>
+        <v>0.7068</v>
       </c>
       <c r="G30" t="n">
         <v>1.7899</v>
       </c>
       <c r="H30" t="n">
-        <v>0.2765</v>
+        <v>0.2632</v>
       </c>
       <c r="I30" t="n">
-        <v>1.86566</v>
+        <v>1.6267</v>
       </c>
       <c r="J30" t="n">
-        <v>0.7235</v>
+        <v>0.7068</v>
       </c>
       <c r="K30" t="n">
         <v>0.08696</v>
       </c>
       <c r="L30" t="n">
-        <v>0.93283</v>
+        <v>0.81335</v>
       </c>
       <c r="M30" t="n">
-        <v>0.86326</v>
+        <v>0.74378</v>
       </c>
       <c r="N30" t="n">
-        <v>1.48</v>
+        <v>2.2</v>
       </c>
       <c r="O30" t="n">
-        <v>1.16</v>
+        <v>1.18</v>
       </c>
       <c r="P30" t="n">
-        <v>1.48</v>
+        <v>2.2</v>
       </c>
       <c r="Q30" t="n">
-        <v>1.16</v>
+        <v>1.18</v>
       </c>
       <c r="R30" t="n">
         <v>0.08699999999999999</v>
       </c>
       <c r="S30" t="n">
-        <v>0.74</v>
+        <v>1.1</v>
       </c>
       <c r="T30" t="n">
-        <v>0.8096</v>
+        <v>1.1696</v>
       </c>
       <c r="U30" t="n">
-        <v>2.54</v>
+        <v>2.6</v>
       </c>
       <c r="V30" t="n">
-        <v>1.5</v>
+        <v>1.25</v>
       </c>
       <c r="W30" t="n">
-        <v>1.38</v>
+        <v>1.42</v>
       </c>
       <c r="X30" t="inlineStr">
         <is>
-          <t>5405-24-20</t>
+          <t>5405-20-32</t>
         </is>
       </c>
       <c r="Y30" t="inlineStr">
         <is>
-          <t>Pipe Adapter (male NPTF x female NPTF), 1 1/2-11 1/2 NPTF x 1 1/4-11 1/2 NPTF (female)</t>
+          <t>Pipe Adapter (male NPTF x female NPTF), 1 1/4-11 1/2 NPTF x 2-11 1/2 NPTF (female)</t>
         </is>
       </c>
       <c r="Z30" t="inlineStr">
@@ -3866,12 +3866,12 @@
       </c>
       <c r="AA30" t="inlineStr">
         <is>
-          <t>1 1/2-11 1/2 NPTF</t>
+          <t>1 1/4-11 1/2 NPTF</t>
         </is>
       </c>
       <c r="AB30" t="inlineStr">
         <is>
-          <t>1 1/4-11 1/2 NPTF (female)</t>
+          <t>2-11 1/2 NPTF (female)</t>
         </is>
       </c>
       <c r="AC30" t="inlineStr">
@@ -3881,34 +3881,34 @@
       </c>
       <c r="AD30" t="inlineStr">
         <is>
-          <t>[BRENNAN-ONLY 2026-10-18] OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); NO Air-Way row for this size -&gt; dimensions MISSING -&gt; 2026-10-18 Brennan allowed (user: "yes use brennan but still differentiate"): L@DRIVE: Brennan TFA catalog p12 table TFA-p012-t02 "5405 MP-FP STRAIGHT EXPANDER" row 5405-24-20 col "L LGTH" = "2.540" (07_RAW_EXTRACTS/brennan_catalogs/TFA Catalog.pdf; brennan_catalog_20261001/catalog_verified.json, line_y 540.0, page verified) [Brennan = yes 2026-10-18] - overall length; mapping: TFA p12 5405 drawing: L = overall, C HEX = body hex, A1 DRILL = male-end bore = SPEC 5405 bore D (impact/F2b.json, certain); same-table check on today's base: 22/28 rows with an Air-Way/OMi value agree with this catalog column to rounding (6 differ, e.g. 5405-08-06 1.87 vs 1.66); CHEX@HEX: Brennan TFA catalog p12 table TFA-p012-t02 "5405 MP-FP STRAIGHT EXPANDER" row 5405-24-20 col "C HEX" = "2.000" (07_RAW_EXTRACTS/brennan_catalogs/TFA Catalog.pdf; brennan_catalog_20261001/catalog_verified.json, line_y 540.0, page verified) [Brennan = yes 2026-10-18] - body hex; mapping: TFA p12 5405 drawing: L = overall, C HEX = body hex, A1 DRILL = male-end bore = SPEC 5405 bore D (impact/F2b.json, certain); same-table check on today's base: 27/28 rows with an Air-Way/OMi value agree with this catalog column to rounding (1 differ, e.g. 5405-08-16 1.38 vs 1.625); D@BORE: Brennan TFA catalog p12 table TFA-p012-t02 "5405 MP-FP STRAIGHT EXPANDER" row 5405-24-20 col "A1 DRILL" = "1.500" (07_RAW_EXTRACTS/brennan_catalogs/TFA Catalog.pdf; brennan_catalog_20261001/catalog_verified.json, line_y 540.0, page verified) [Brennan = yes 2026-10-18] - male-end bore (to the pocket); mapping: TFA p12 5405 drawing: L = overall, C HEX = body hex, A1 DRILL = male-end bore = SPEC 5405 bore D (impact/F2b.json, certain); same-table check on today's base: 27/28 rows with an Air-Way/OMi value agree with this catalog column to rounding (1 differ, e.g. 5405-16-08 0.94 vs 0.697); TAPDRILL@BORE: end library gen_straight2 FPT[20] (= tools_new/generators/templates/DesignTable_2405_SW2.xlsx row of that pipe dash: TAPDRILL@BORE_A 1.48, FPT_P1 1.16 = MS51503 P1 max) = Air-Way per-size tap drill (-02 0.33 ... -20 1.48) [user 2026-10-18 A1 Q-TRANSFER-TAPDRILL yes, 00_DOCS/ANSWERS_2026-10-18.md]; THDMAJ_A1@DRIVE: end library: ASME B1.20.1 / B1.20.3 1-1/2 NPT basic dimensions = tools_new/generators/ms51500.NPTF[24] [Q-TRANSFER-ENDLIB yes 2026-10-08] pipe OD (male end); THDMAJ_A2@DRIVE: end library: ASME B1.20.1 / B1.20.3 1-1/4 NPT basic dimensions = tools_new/generators/ms51500.NPTF[20] [Q-TRANSFER-ENDLIB yes 2026-10-08] pipe OD (female end); $PRP@Threads: thread texts from the part-number dashes, format of the built 5405 rows | MODEL: NPTF male end per ASME B1.20.3 with the 5404 Brennan-measured end length for the same dash (ASSUMPTION); female drill depth = MS51503 P1 max per pipe dash (2405 table), thread cut to full drill depth (ASSUMPTION); Brennan 5405-08-08 STEP (2026-09-23) confirms 1/2 NPTF port drill depth 0.900 = MS51503 P1 max (VERIFIED for -08 only; thread taper depth in that STEP is 0.750, tap drill dia 0.718, drill point 120 deg); bore D runs from the male tip to the pocket bottom</t>
+          <t>[A1/A9 TAPDRILL 2026-10-21: TAPDRILL@BORE] [BRENNAN-CAD 2026-10-21: CHEX@HEX, D@BORE, L@DRIVE, THDMAJ_A1@DRIVE, THDMAJ_A2@DRIVE] OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); NO Air-Way row for this size -&gt; dimensions MISSING | MODEL: NPTF male end per ASME B1.20.3 with the 5404 Brennan-measured end length for the same dash (ASSUMPTION); female drill depth = MS51503 P1 max per pipe dash (2405 table), thread cut to full drill depth (ASSUMPTION); Brennan 5405-08-08 STEP (2026-09-23) confirms 1/2 NPTF port drill depth 0.900 = MS51503 P1 max (VERIFIED for -08 only; thread taper depth in that STEP is 0.750, tap drill dia 0.718, drill point 120 deg); bore D runs from the male tip to the pocket bottom</t>
         </is>
       </c>
       <c r="AE30" t="inlineStr">
         <is>
-          <t>BUILD-MISSING: part exists in OMi catalog but the Air-Way page has no row; needs a second dimensional source | 2026-10-18 Brennan = yes (wave 2 straight, staged, not shipped): L / hex / D from the Brennan TFA catalog p12 alone; tap drill = Air-Way per size (A1 yes) | ASSUMPTION: Air-Way bore D 1.5 is wider than the port tap drill 1.48 - the bore stops at the port bottom, leaving a 0.010 internal step there (real part unconfirmed)</t>
+          <t>BUILD-MISSING: part exists in OMi catalog but the Air-Way page has no row; needs a second dimensional source | Brennan CAD record 5405-20-32 (PARTcommunity / CADENAS, CHEX@HEX=C, D@BORE=A1D, L@DRIVE=L, THDMAJ_A1@DRIVE=A1THD, THDMAJ_A2@DRIVE=A2THD; user 2026-10-21 "yes you can use them following my rule") | TAPDRILL@BORE = Air-Way per-size tap drill -32 2.2 (A1, A9: Brennan 5405-24-24 / -32-32 STEPs 1.734 / 2.218 -&gt; nearest Air-Way 1.72 / 2.20)</t>
         </is>
       </c>
       <c r="AF30" t="inlineStr">
         <is>
-          <t>5405-24-20</t>
+          <t>5405-20-32</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>5405-24-24</t>
+          <t>5405-24-20</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>2.53</v>
+        <v>2.54</v>
       </c>
       <c r="C31" t="n">
-        <v>1.37409</v>
+        <v>1.1547</v>
       </c>
       <c r="D31" t="n">
-        <v>2.38</v>
+        <v>2</v>
       </c>
       <c r="E31" t="n">
         <v>0.93283</v>
@@ -3938,13 +3938,13 @@
         <v>0.86326</v>
       </c>
       <c r="N31" t="n">
-        <v>1.72</v>
+        <v>1.48</v>
       </c>
       <c r="O31" t="n">
         <v>1.16</v>
       </c>
       <c r="P31" t="n">
-        <v>1.72</v>
+        <v>1.48</v>
       </c>
       <c r="Q31" t="n">
         <v>1.16</v>
@@ -3953,28 +3953,28 @@
         <v>0.08699999999999999</v>
       </c>
       <c r="S31" t="n">
-        <v>0.86</v>
+        <v>0.74</v>
       </c>
       <c r="T31" t="n">
-        <v>0.9296</v>
+        <v>0.8096</v>
       </c>
       <c r="U31" t="n">
-        <v>2.53</v>
+        <v>2.54</v>
       </c>
       <c r="V31" t="n">
         <v>1.5</v>
       </c>
       <c r="W31" t="n">
-        <v>1.37</v>
+        <v>1.38</v>
       </c>
       <c r="X31" t="inlineStr">
         <is>
-          <t>5405-24-24</t>
+          <t>5405-24-20</t>
         </is>
       </c>
       <c r="Y31" t="inlineStr">
         <is>
-          <t>Pipe Adapter (male NPTF x female NPTF), 1 1/2-11 1/2 NPTF x 1 1/2-11 1/2 NPTF (female)</t>
+          <t>Pipe Adapter (male NPTF x female NPTF), 1 1/2-11 1/2 NPTF x 1 1/4-11 1/2 NPTF (female)</t>
         </is>
       </c>
       <c r="Z31" t="inlineStr">
@@ -3989,7 +3989,7 @@
       </c>
       <c r="AB31" t="inlineStr">
         <is>
-          <t>1 1/2-11 1/2 NPTF (female)</t>
+          <t>1 1/4-11 1/2 NPTF (female)</t>
         </is>
       </c>
       <c r="AC31" t="inlineStr">
@@ -3999,29 +3999,34 @@
       </c>
       <c r="AD31" t="inlineStr">
         <is>
-          <t>Air-Way s85 only (no MS sheet exists for this topology); double-pass 28 rows | MODEL: NPTF male end per ASME B1.20.3 with the 5404 Brennan-measured end length for the same dash (ASSUMPTION); female drill depth = MS51503 P1 max per pipe dash (2405 table), thread cut to full drill depth (ASSUMPTION); Brennan 5405-08-08 STEP (2026-09-23) confirms 1/2 NPTF port drill depth 0.900 = MS51503 P1 max (VERIFIED for -08 only; thread taper depth in that STEP is 0.750, tap drill dia 0.718, drill point 120 deg); bore D runs from the male tip to the pocket bottom</t>
+          <t>[BRENNAN-ONLY 2026-10-18] OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); NO Air-Way row for this size -&gt; dimensions MISSING -&gt; 2026-10-18 Brennan allowed (user: "yes use brennan but still differentiate"): L@DRIVE: Brennan TFA catalog p12 table TFA-p012-t02 "5405 MP-FP STRAIGHT EXPANDER" row 5405-24-20 col "L LGTH" = "2.540" (07_RAW_EXTRACTS/brennan_catalogs/TFA Catalog.pdf; brennan_catalog_20261001/catalog_verified.json, line_y 540.0, page verified) [Brennan = yes 2026-10-18] - overall length; mapping: TFA p12 5405 drawing: L = overall, C HEX = body hex, A1 DRILL = male-end bore = SPEC 5405 bore D (impact/F2b.json, certain); same-table check on today's base: 22/28 rows with an Air-Way/OMi value agree with this catalog column to rounding (6 differ, e.g. 5405-08-06 1.87 vs 1.66); CHEX@HEX: Brennan TFA catalog p12 table TFA-p012-t02 "5405 MP-FP STRAIGHT EXPANDER" row 5405-24-20 col "C HEX" = "2.000" (07_RAW_EXTRACTS/brennan_catalogs/TFA Catalog.pdf; brennan_catalog_20261001/catalog_verified.json, line_y 540.0, page verified) [Brennan = yes 2026-10-18] - body hex; mapping: TFA p12 5405 drawing: L = overall, C HEX = body hex, A1 DRILL = male-end bore = SPEC 5405 bore D (impact/F2b.json, certain); same-table check on today's base: 27/28 rows with an Air-Way/OMi value agree with this catalog column to rounding (1 differ, e.g. 5405-08-16 1.38 vs 1.625); D@BORE: Brennan TFA catalog p12 table TFA-p012-t02 "5405 MP-FP STRAIGHT EXPANDER" row 5405-24-20 col "A1 DRILL" = "1.500" (07_RAW_EXTRACTS/brennan_catalogs/TFA Catalog.pdf; brennan_catalog_20261001/catalog_verified.json, line_y 540.0, page verified) [Brennan = yes 2026-10-18] - male-end bore (to the pocket); mapping: TFA p12 5405 drawing: L = overall, C HEX = body hex, A1 DRILL = male-end bore = SPEC 5405 bore D (impact/F2b.json, certain); same-table check on today's base: 27/28 rows with an Air-Way/OMi value agree with this catalog column to rounding (1 differ, e.g. 5405-16-08 0.94 vs 0.697); TAPDRILL@BORE: end library gen_straight2 FPT[20] (= tools_new/generators/templates/DesignTable_2405_SW2.xlsx row of that pipe dash: TAPDRILL@BORE_A 1.48, FPT_P1 1.16 = MS51503 P1 max) = Air-Way per-size tap drill (-02 0.33 ... -20 1.48) [user 2026-10-18 A1 Q-TRANSFER-TAPDRILL yes, 00_DOCS/ANSWERS_2026-10-18.md]; THDMAJ_A1@DRIVE: end library: ASME B1.20.1 / B1.20.3 1-1/2 NPT basic dimensions = tools_new/generators/ms51500.NPTF[24] [Q-TRANSFER-ENDLIB yes 2026-10-08] pipe OD (male end); THDMAJ_A2@DRIVE: end library: ASME B1.20.1 / B1.20.3 1-1/4 NPT basic dimensions = tools_new/generators/ms51500.NPTF[20] [Q-TRANSFER-ENDLIB yes 2026-10-08] pipe OD (female end); $PRP@Threads: thread texts from the part-number dashes, format of the built 5405 rows | MODEL: NPTF male end per ASME B1.20.3 with the 5404 Brennan-measured end length for the same dash (ASSUMPTION); female drill depth = MS51503 P1 max per pipe dash (2405 table), thread cut to full drill depth (ASSUMPTION); Brennan 5405-08-08 STEP (2026-09-23) confirms 1/2 NPTF port drill depth 0.900 = MS51503 P1 max (VERIFIED for -08 only; thread taper depth in that STEP is 0.750, tap drill dia 0.718, drill point 120 deg); bore D runs from the male tip to the pocket bottom</t>
+        </is>
+      </c>
+      <c r="AE31" t="inlineStr">
+        <is>
+          <t>BUILD-MISSING: part exists in OMi catalog but the Air-Way page has no row; needs a second dimensional source | 2026-10-18 Brennan = yes (wave 2 straight, staged, not shipped): L / hex / D from the Brennan TFA catalog p12 alone; tap drill = Air-Way per size (A1 yes) | ASSUMPTION: Air-Way bore D 1.5 is wider than the port tap drill 1.48 - the bore stops at the port bottom, leaving a 0.010 internal step there (real part unconfirmed)</t>
         </is>
       </c>
       <c r="AF31" t="inlineStr">
         <is>
-          <t>5405-24-24</t>
+          <t>5405-24-20</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>5405-24-32</t>
+          <t>5405-24-24</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>2.63</v>
+        <v>2.53</v>
       </c>
       <c r="C32" t="n">
-        <v>1.66277</v>
+        <v>1.37409</v>
       </c>
       <c r="D32" t="n">
-        <v>2.88</v>
+        <v>2.38</v>
       </c>
       <c r="E32" t="n">
         <v>0.93283</v>
@@ -4051,43 +4056,43 @@
         <v>0.86326</v>
       </c>
       <c r="N32" t="n">
-        <v>2.19</v>
+        <v>1.72</v>
       </c>
       <c r="O32" t="n">
-        <v>1.18</v>
+        <v>1.16</v>
       </c>
       <c r="P32" t="n">
-        <v>2.19</v>
+        <v>1.72</v>
       </c>
       <c r="Q32" t="n">
-        <v>1.18</v>
+        <v>1.16</v>
       </c>
       <c r="R32" t="n">
         <v>0.08699999999999999</v>
       </c>
       <c r="S32" t="n">
-        <v>1.095</v>
+        <v>0.86</v>
       </c>
       <c r="T32" t="n">
-        <v>1.1646</v>
+        <v>0.9296</v>
       </c>
       <c r="U32" t="n">
-        <v>2.63</v>
+        <v>2.53</v>
       </c>
       <c r="V32" t="n">
         <v>1.5</v>
       </c>
       <c r="W32" t="n">
-        <v>1.45</v>
+        <v>1.37</v>
       </c>
       <c r="X32" t="inlineStr">
         <is>
-          <t>5405-24-32</t>
+          <t>5405-24-24</t>
         </is>
       </c>
       <c r="Y32" t="inlineStr">
         <is>
-          <t>Pipe Adapter (male NPTF x female NPTF), 1 1/2-11 1/2 NPTF x 2-11 1/2 NPTF (female)</t>
+          <t>Pipe Adapter (male NPTF x female NPTF), 1 1/2-11 1/2 NPTF x 1 1/2-11 1/2 NPTF (female)</t>
         </is>
       </c>
       <c r="Z32" t="inlineStr">
@@ -4102,7 +4107,7 @@
       </c>
       <c r="AB32" t="inlineStr">
         <is>
-          <t>2-11 1/2 NPTF (female)</t>
+          <t>1 1/2-11 1/2 NPTF (female)</t>
         </is>
       </c>
       <c r="AC32" t="inlineStr">
@@ -4117,18 +4122,18 @@
       </c>
       <c r="AF32" t="inlineStr">
         <is>
-          <t>5405-24-32</t>
+          <t>5405-24-24</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>5405-32-32</t>
+          <t>5405-24-32</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>2.66</v>
+        <v>2.63</v>
       </c>
       <c r="C33" t="n">
         <v>1.66277</v>
@@ -4137,40 +4142,40 @@
         <v>2.88</v>
       </c>
       <c r="E33" t="n">
-        <v>1.16929</v>
+        <v>0.93283</v>
       </c>
       <c r="F33" t="n">
-        <v>0.7565</v>
+        <v>0.7235</v>
       </c>
       <c r="G33" t="n">
         <v>1.7899</v>
       </c>
       <c r="H33" t="n">
-        <v>0.2735</v>
+        <v>0.2765</v>
       </c>
       <c r="I33" t="n">
-        <v>2.33859</v>
+        <v>1.86566</v>
       </c>
       <c r="J33" t="n">
-        <v>0.7565</v>
+        <v>0.7235</v>
       </c>
       <c r="K33" t="n">
         <v>0.08696</v>
       </c>
       <c r="L33" t="n">
-        <v>1.16929</v>
+        <v>0.93283</v>
       </c>
       <c r="M33" t="n">
-        <v>1.09973</v>
+        <v>0.86326</v>
       </c>
       <c r="N33" t="n">
-        <v>2.2</v>
+        <v>2.19</v>
       </c>
       <c r="O33" t="n">
         <v>1.18</v>
       </c>
       <c r="P33" t="n">
-        <v>2.2</v>
+        <v>2.19</v>
       </c>
       <c r="Q33" t="n">
         <v>1.18</v>
@@ -4179,61 +4184,174 @@
         <v>0.08699999999999999</v>
       </c>
       <c r="S33" t="n">
+        <v>1.095</v>
+      </c>
+      <c r="T33" t="n">
+        <v>1.1646</v>
+      </c>
+      <c r="U33" t="n">
+        <v>2.63</v>
+      </c>
+      <c r="V33" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="W33" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="X33" t="inlineStr">
+        <is>
+          <t>5405-24-32</t>
+        </is>
+      </c>
+      <c r="Y33" t="inlineStr">
+        <is>
+          <t>Pipe Adapter (male NPTF x female NPTF), 1 1/2-11 1/2 NPTF x 2-11 1/2 NPTF (female)</t>
+        </is>
+      </c>
+      <c r="Z33" t="inlineStr">
+        <is>
+          <t>5405</t>
+        </is>
+      </c>
+      <c r="AA33" t="inlineStr">
+        <is>
+          <t>1 1/2-11 1/2 NPTF</t>
+        </is>
+      </c>
+      <c r="AB33" t="inlineStr">
+        <is>
+          <t>2-11 1/2 NPTF (female)</t>
+        </is>
+      </c>
+      <c r="AC33" t="inlineStr">
+        <is>
+          <t>ASSUMED</t>
+        </is>
+      </c>
+      <c r="AD33" t="inlineStr">
+        <is>
+          <t>Air-Way s85 only (no MS sheet exists for this topology); double-pass 28 rows | MODEL: NPTF male end per ASME B1.20.3 with the 5404 Brennan-measured end length for the same dash (ASSUMPTION); female drill depth = MS51503 P1 max per pipe dash (2405 table), thread cut to full drill depth (ASSUMPTION); Brennan 5405-08-08 STEP (2026-09-23) confirms 1/2 NPTF port drill depth 0.900 = MS51503 P1 max (VERIFIED for -08 only; thread taper depth in that STEP is 0.750, tap drill dia 0.718, drill point 120 deg); bore D runs from the male tip to the pocket bottom</t>
+        </is>
+      </c>
+      <c r="AF33" t="inlineStr">
+        <is>
+          <t>5405-24-32</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>5405-32-32</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>2.66</v>
+      </c>
+      <c r="C34" t="n">
+        <v>1.66277</v>
+      </c>
+      <c r="D34" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="E34" t="n">
+        <v>1.16929</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0.7565</v>
+      </c>
+      <c r="G34" t="n">
+        <v>1.7899</v>
+      </c>
+      <c r="H34" t="n">
+        <v>0.2735</v>
+      </c>
+      <c r="I34" t="n">
+        <v>2.33859</v>
+      </c>
+      <c r="J34" t="n">
+        <v>0.7565</v>
+      </c>
+      <c r="K34" t="n">
+        <v>0.08696</v>
+      </c>
+      <c r="L34" t="n">
+        <v>1.16929</v>
+      </c>
+      <c r="M34" t="n">
+        <v>1.09973</v>
+      </c>
+      <c r="N34" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="O34" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="P34" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="Q34" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="R34" t="n">
+        <v>0.08699999999999999</v>
+      </c>
+      <c r="S34" t="n">
         <v>1.1</v>
       </c>
-      <c r="T33" t="n">
+      <c r="T34" t="n">
         <v>1.1696</v>
       </c>
-      <c r="U33" t="n">
+      <c r="U34" t="n">
         <v>2.66</v>
       </c>
-      <c r="V33" t="n">
+      <c r="V34" t="n">
         <v>1.94</v>
       </c>
-      <c r="W33" t="n">
+      <c r="W34" t="n">
         <v>1.48</v>
       </c>
-      <c r="X33" t="inlineStr">
+      <c r="X34" t="inlineStr">
         <is>
           <t>5405-32-32</t>
         </is>
       </c>
-      <c r="Y33" t="inlineStr">
+      <c r="Y34" t="inlineStr">
         <is>
           <t>Pipe Adapter (male NPTF x female NPTF), 2-11 1/2 NPTF x 2-11 1/2 NPTF (female)</t>
         </is>
       </c>
-      <c r="Z33" t="inlineStr">
+      <c r="Z34" t="inlineStr">
         <is>
           <t>5405</t>
         </is>
       </c>
-      <c r="AA33" t="inlineStr">
+      <c r="AA34" t="inlineStr">
         <is>
           <t>2-11 1/2 NPTF</t>
         </is>
       </c>
-      <c r="AB33" t="inlineStr">
+      <c r="AB34" t="inlineStr">
         <is>
           <t>2-11 1/2 NPTF (female)</t>
         </is>
       </c>
-      <c r="AC33" t="inlineStr">
+      <c r="AC34" t="inlineStr">
         <is>
           <t>ASSUMED</t>
         </is>
       </c>
-      <c r="AD33" t="inlineStr">
+      <c r="AD34" t="inlineStr">
         <is>
           <t>Air-Way s85 only (no MS sheet exists for this topology); double-pass 28 rows | MODEL: NPTF male end per ASME B1.20.3 with the 5404 Brennan-measured end length for the same dash (ASSUMPTION); female drill depth = MS51503 P1 max per pipe dash (2405 table), thread cut to full drill depth (ASSUMPTION); Brennan 5405-08-08 STEP (2026-09-23) confirms 1/2 NPTF port drill depth 0.900 = MS51503 P1 max (VERIFIED for -08 only; thread taper depth in that STEP is 0.750, tap drill dia 0.718, drill point 120 deg); bore D runs from the male tip to the pocket bottom</t>
         </is>
       </c>
-      <c r="AE33" t="inlineStr">
+      <c r="AE34" t="inlineStr">
         <is>
           <t>tap drill printed 2.20 (24-32 row prints 2.19 for same 2-11 1/2 thread) - as-printed</t>
         </is>
       </c>
-      <c r="AF33" t="inlineStr">
+      <c r="AF34" t="inlineStr">
         <is>
           <t>5405-32-32</t>
         </is>

</xml_diff>